<commit_message>
feat(resultados): liquidacao oficial de 22 jogos e nova pagina 05 de resultados forward
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
@@ -558,15 +558,19 @@
       <c r="K2" t="n">
         <v>2.48</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -626,15 +630,19 @@
       <c r="K3" t="n">
         <v>2.06</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -694,15 +702,19 @@
       <c r="K4" t="n">
         <v>2.06</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -762,15 +774,19 @@
       <c r="K5" t="n">
         <v>1.28</v>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -830,15 +846,19 @@
       <c r="K6" t="n">
         <v>1.41</v>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -898,15 +918,19 @@
       <c r="K7" t="n">
         <v>1.29</v>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -966,15 +990,19 @@
       <c r="K8" t="n">
         <v>1.24</v>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>AO Away Win</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1034,15 +1062,19 @@
       <c r="K9" t="n">
         <v>1.4</v>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1102,15 +1134,19 @@
       <c r="K10" t="n">
         <v>2.6</v>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1170,15 +1206,19 @@
       <c r="K11" t="n">
         <v>1.29</v>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>AO Home Win</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1238,15 +1278,19 @@
       <c r="K12" t="n">
         <v>1.65</v>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1306,15 +1350,19 @@
       <c r="K13" t="n">
         <v>1.5</v>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1374,15 +1422,19 @@
       <c r="K14" t="n">
         <v>1.26</v>
       </c>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1442,15 +1494,19 @@
       <c r="K15" t="n">
         <v>2.06</v>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1510,15 +1566,19 @@
       <c r="K16" t="n">
         <v>2.06</v>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1578,15 +1638,19 @@
       <c r="K17" t="n">
         <v>1.58</v>
       </c>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1646,15 +1710,19 @@
       <c r="K18" t="n">
         <v>1.58</v>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1714,15 +1782,19 @@
       <c r="K19" t="n">
         <v>1.59</v>
       </c>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1782,15 +1854,19 @@
       <c r="K20" t="n">
         <v>1.59</v>
       </c>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1850,15 +1926,19 @@
       <c r="K21" t="n">
         <v>2.38</v>
       </c>
-      <c r="L21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1918,15 +1998,19 @@
       <c r="K22" t="n">
         <v>1.36</v>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1986,15 +2070,19 @@
       <c r="K23" t="n">
         <v>1.58</v>
       </c>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">

</xml_diff>

<commit_message>
feat(portfolio): expurgamento definitivo do metodo Lay 0x3 do operacional ativo e Streamlit
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -595,27 +595,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Indonesian Championship</t>
+          <t>Thai League 3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Persiku Kudus x Psgc Ciamis</t>
+          <t>Prime Bangkok x Lopburi City FC</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Persiku Kudus</t>
+          <t>Prime Bangkok</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Psgc Ciamis</t>
+          <t>Lopburi City FC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lay 0x3 (Regra Ampla)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -625,14 +625,14 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>30</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>2.06</v>
+        <v>1.28</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>71</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4">
@@ -667,27 +667,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Indonesian Championship</t>
+          <t>Thai League 3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Persiku Kudus x Psgc Ciamis</t>
+          <t>Udon Banjan United x Korat City</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Persiku Kudus</t>
+          <t>Udon Banjan United</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Psgc Ciamis</t>
+          <t>Korat City</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -697,14 +697,14 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="K4" t="n">
-        <v>2.06</v>
+        <v>1.41</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -734,27 +734,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thai League 3</t>
+          <t>Norwegian 2nd Division</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Prime Bangkok x Lopburi City FC</t>
+          <t>Ullensaker Kisa x Kjelsas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Prime Bangkok</t>
+          <t>Ullensaker Kisa</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Lopburi City FC</t>
+          <t>Kjelsas</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -769,14 +769,14 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>8.800000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="K5" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>205</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6">
@@ -806,32 +806,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thai League 3</t>
+          <t>Estonian Cup</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Udon Banjan United x Korat City</t>
+          <t>FC Tallinn x Harju JK Laagri</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Udon Banjan United</t>
+          <t>FC Tallinn</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Korat City</t>
+          <t>Harju JK Laagri</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -841,14 +841,14 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>18</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>1.41</v>
+        <v>1.24</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>AO Away Win</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7">
@@ -878,7 +878,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -888,17 +888,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ullensaker Kisa x Kjelsas</t>
+          <t>Notodden x Eik-Tonsberg</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Ullensaker Kisa</t>
+          <t>Notodden</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Kjelsas</t>
+          <t>Eik-Tonsberg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -913,14 +913,14 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>7.8</v>
+        <v>6</v>
       </c>
       <c r="K7" t="n">
-        <v>1.29</v>
+        <v>1.4</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>185</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8">
@@ -950,32 +950,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Estonian Cup</t>
+          <t>English Sky Bet League 2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FC Tallinn x Harju JK Laagri</t>
+          <t>Exeter x Rotherham</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FC Tallinn</t>
+          <t>Exeter</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Harju JK Laagri</t>
+          <t>Rotherham</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -985,14 +985,14 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>8.199999999999999</v>
+        <v>16.5</v>
       </c>
       <c r="K8" t="n">
-        <v>1.24</v>
+        <v>2.6</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>AO Away Win</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>85</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9">
@@ -1022,27 +1022,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Norwegian 2nd Division</t>
+          <t>Scottish League One</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Notodden x Eik-Tonsberg</t>
+          <t>Ross Co x Alloa</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Notodden</t>
+          <t>Ross Co</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Eik-Tonsberg</t>
+          <t>Alloa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1057,14 +1057,14 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9" t="n">
-        <v>1.4</v>
+        <v>1.29</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>AO Home Win</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>167</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10">
@@ -1099,27 +1099,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>English Sky Bet League 2</t>
+          <t>Scottish Championship</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exeter x Rotherham</t>
+          <t>Morton x Raith</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Exeter</t>
+          <t>Morton</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Rotherham</t>
+          <t>Raith</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1129,14 +1129,14 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>16.5</v>
+        <v>6.4</v>
       </c>
       <c r="K10" t="n">
-        <v>2.6</v>
+        <v>1.65</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>229</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11">
@@ -1171,27 +1171,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Scottish League One</t>
+          <t>English National League</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ross Co x Alloa</t>
+          <t>Gateshead x Worthing</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ross Co</t>
+          <t>Gateshead</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Alloa</t>
+          <t>Worthing</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1201,14 +1201,14 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="K11" t="n">
-        <v>1.29</v>
+        <v>1.5</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>AO Home Win</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12">
@@ -1243,27 +1243,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Scottish Championship</t>
+          <t>Algerian Ligue 2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Morton x Raith</t>
+          <t>USM El Harrach x Taghit</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Morton</t>
+          <t>USM El Harrach</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Raith</t>
+          <t>Taghit</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1273,14 +1273,14 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>6.4</v>
+        <v>15</v>
       </c>
       <c r="K12" t="n">
-        <v>1.65</v>
+        <v>1.26</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>4-0</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>159</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13">
@@ -1310,32 +1310,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>English National League</t>
+          <t>German Frauen-Bundesliga</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Gateshead x Worthing</t>
+          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Gateshead</t>
+          <t>Eintracht Frankfurt (W)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Worthing</t>
+          <t>Bayern Munich (W)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1345,14 +1345,14 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>7.2</v>
+        <v>18</v>
       </c>
       <c r="K13" t="n">
-        <v>1.5</v>
+        <v>1.58</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>231</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14">
@@ -1382,32 +1382,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Algerian Ligue 2</t>
+          <t>German Frauen-Bundesliga</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>USM El Harrach x Taghit</t>
+          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>USM El Harrach</t>
+          <t>Eintracht Frankfurt (W)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Taghit</t>
+          <t>Bayern Munich (W)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1417,14 +1417,14 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="K14" t="n">
-        <v>1.26</v>
+        <v>1.58</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15">
@@ -1454,32 +1454,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chilean Tercera Division</t>
+          <t>Guatemalan Liga Nacional</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Chimbarongo FC x Club Malleco Unido</t>
+          <t>Deportivo Mixco x CSD Municipal</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Chimbarongo FC</t>
+          <t>Deportivo Mixco</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Club Malleco Unido</t>
+          <t>CSD Municipal</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Lay 0x3 (Regra Ampla)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1489,19 +1489,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>27</v>
+        <v>17.5</v>
       </c>
       <c r="K15" t="n">
-        <v>2.06</v>
+        <v>2.38</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16">
@@ -1526,32 +1526,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chilean Tercera Division</t>
+          <t>UEFA Nations League B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Chimbarongo FC x Club Malleco Unido</t>
+          <t>Switzerland x Slovenia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Chimbarongo FC</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Club Malleco Unido</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1561,19 +1561,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>27</v>
+        <v>5.5</v>
       </c>
       <c r="K16" t="n">
-        <v>2.06</v>
+        <v>1.36</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>136</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17">
@@ -1598,32 +1598,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>German Frauen-Bundesliga</t>
+          <t>UEFA Nations League B</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
+          <t>North Macedonia x Scotland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W)</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bayern Munich (W)</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>18</v>
+        <v>8.6</v>
       </c>
       <c r="K17" t="n">
         <v>1.58</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>95</v>
+        <v>2784</v>
       </c>
     </row>
     <row r="18">
@@ -1670,32 +1670,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>German Frauen-Bundesliga</t>
+          <t>Brazilian Serie B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
+          <t>Cuiaba x Ponte Preta</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W)</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bayern Munich (W)</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1705,24 +1705,20 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
+        <v>1.16</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>✅ LIQUIDADO</t>
+          <t>⏳ PENDENTE</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1731,7 +1727,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19">
@@ -1742,32 +1738,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Moroccan Botola Pro 1</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HUSA Agadir x MAS Maghrib A Fes</t>
+          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HUSA Agadir</t>
+          <t>CSD Liniers de Ciudad Evita</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MAS Maghrib A Fes</t>
+          <t>Excursionistas</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lay 0x3 (Regra Ampla)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1777,24 +1773,20 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
+        <v>1.01</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>✅ LIQUIDADO</t>
+          <t>⏳ PENDENTE</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1803,7 +1795,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>86</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20">
@@ -1814,32 +1806,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Moroccan Botola Pro 1</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>HUSA Agadir x MAS Maghrib A Fes</t>
+          <t>Camioneros x Deportivo Laferrere</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HUSA Agadir</t>
+          <t>Camioneros</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>MAS Maghrib A Fes</t>
+          <t>Deportivo Laferrere</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1849,24 +1841,20 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>30</v>
+        <v>6.6</v>
       </c>
       <c r="K20" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
+        <v>1.23</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>✅ LIQUIDADO</t>
+          <t>⏳ PENDENTE</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1875,7 +1863,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>86</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21">
@@ -1886,32 +1874,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Guatemalan Liga Nacional</t>
+          <t>Brazilian Serie C</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Deportivo Mixco x CSD Municipal</t>
+          <t>Floresta EC x Botafogo PB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Deportivo Mixco</t>
+          <t>Floresta EC</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CSD Municipal</t>
+          <t>Botafogo PB</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1921,24 +1909,20 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>17.5</v>
+        <v>19.5</v>
       </c>
       <c r="K21" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+        <v>1.48</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>✅ LIQUIDADO</t>
+          <t>⏳ PENDENTE</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1947,7 +1931,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>141</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22">
@@ -1958,32 +1942,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>UEFA Nations League B</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Switzerland x Slovenia</t>
+          <t>Camioneros x Deportivo Laferrere</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Camioneros</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Deportivo Laferrere</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1993,24 +1977,20 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>5.5</v>
+        <v>18</v>
       </c>
       <c r="K22" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2-1</t>
-        </is>
-      </c>
+        <v>1.02</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>✅ LIQUIDADO</t>
+          <t>⏳ PENDENTE</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2019,418 +1999,6 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>UEFA Nations League B</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>North Macedonia x Scotland</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>North Macedonia</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Scotland</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="K23" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>✅ LIQUIDADO</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>2784</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Brazilian Serie B</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Cuiaba x Ponte Preta</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Cuiaba</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Ponte Preta</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Argentinian Primera B Metropolitana</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>CSD Liniers de Ciudad Evita</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Excursionistas</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>5</v>
-      </c>
-      <c r="K25" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Argentinian Primera B Metropolitana</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Camioneros x Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Camioneros</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="K26" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Brazilian Serie C</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Floresta EC x Botafogo PB</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Floresta EC</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Botafogo PB</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="K27" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Argentinian Primera B Metropolitana</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Camioneros x Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Camioneros</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>18</v>
-      </c>
-      <c r="K28" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(radar): atualizar grade com jogos noturnos 18h05 e 18h15 (23 jogos)
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2002,6 +2002,142 @@
         <v>92</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Colombian Primera A</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tolima x Boyaca Chico</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Boyaca Chico</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bolivian Cup</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Nacional Potosi x CDT Real Oruro</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Nacional Potosi</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CDT Real Oruro</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(resultados): refazer e liquidar resultados oficiais de 03/10 e 04/10 com filtros estritos de ligas
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T24"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,26 +509,6 @@
           <t>Liquidez_Lay</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Hora_Str</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Risco_Red_R$</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Stake_Sugerida_R$</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Lucro_Green_R$</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -538,32 +518,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Japanese J League 3</t>
+          <t>Norwegian 2nd Division</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kitakyushu x Kochi United</t>
+          <t>Ullensaker Kisa x Kjelsas</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Kitakyushu</t>
+          <t>Ullensaker Kisa</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Kochi United</t>
+          <t>Kjelsas</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -573,14 +553,14 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>18</v>
+        <v>7.8</v>
       </c>
       <c r="K2" t="n">
-        <v>2.48</v>
+        <v>1.29</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -599,21 +579,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>169</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>05:00</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>200</v>
-      </c>
-      <c r="S2" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="T2" t="n">
-        <v>11.23</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3">
@@ -624,27 +590,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thai League 3</t>
+          <t>Norwegian 2nd Division</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Prime Bangkok x Lopburi City FC</t>
+          <t>Notodden x Eik-Tonsberg</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Prime Bangkok</t>
+          <t>Notodden</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Lopburi City FC</t>
+          <t>Eik-Tonsberg</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -659,14 +625,14 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>8.800000000000001</v>
+        <v>6</v>
       </c>
       <c r="K3" t="n">
-        <v>1.28</v>
+        <v>1.4</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -685,21 +651,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>205</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>05:30</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>200</v>
-      </c>
-      <c r="S3" t="n">
-        <v>25.64</v>
-      </c>
-      <c r="T3" t="n">
-        <v>24.49</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
@@ -710,32 +662,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thai League 3</t>
+          <t>English Sky Bet League 2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Udon Banjan United x Korat City</t>
+          <t>Exeter x Rotherham</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Udon Banjan United</t>
+          <t>Exeter</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Korat City</t>
+          <t>Rotherham</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -745,14 +697,14 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>18</v>
+        <v>16.5</v>
       </c>
       <c r="K4" t="n">
-        <v>1.41</v>
+        <v>2.6</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -771,21 +723,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>78</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>05:30</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>200</v>
-      </c>
-      <c r="S4" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="T4" t="n">
-        <v>11.23</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5">
@@ -796,27 +734,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Norwegian 2nd Division</t>
+          <t>Scottish League One</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ullensaker Kisa x Kjelsas</t>
+          <t>Ross Co x Alloa</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ullensaker Kisa</t>
+          <t>Ross Co</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Kjelsas</t>
+          <t>Alloa</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -831,14 +769,14 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
         <v>1.29</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>AO Home Win</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -857,21 +795,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>185</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>200</v>
-      </c>
-      <c r="S5" t="n">
-        <v>29.41</v>
-      </c>
-      <c r="T5" t="n">
-        <v>28.09</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6">
@@ -882,32 +806,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Estonian Cup</t>
+          <t>Scottish Championship</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FC Tallinn x Harju JK Laagri</t>
+          <t>Morton x Raith</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FC Tallinn</t>
+          <t>Morton</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Harju JK Laagri</t>
+          <t>Raith</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -917,14 +841,14 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>8.199999999999999</v>
+        <v>6.4</v>
       </c>
       <c r="K6" t="n">
-        <v>1.24</v>
+        <v>1.65</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>AO Away Win</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -943,21 +867,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>85</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>200</v>
-      </c>
-      <c r="S6" t="n">
-        <v>27.78</v>
-      </c>
-      <c r="T6" t="n">
-        <v>26.53</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7">
@@ -968,32 +878,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Norwegian 2nd Division</t>
+          <t>English National League</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Notodden x Eik-Tonsberg</t>
+          <t>Gateshead x Worthing</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Notodden</t>
+          <t>Gateshead</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Eik-Tonsberg</t>
+          <t>Worthing</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1003,14 +913,14 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>6</v>
+        <v>7.2</v>
       </c>
       <c r="K7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1029,21 +939,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>167</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="R7" t="n">
-        <v>200</v>
-      </c>
-      <c r="S7" t="n">
-        <v>40</v>
-      </c>
-      <c r="T7" t="n">
-        <v>38.2</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8">
@@ -1059,27 +955,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>English Sky Bet League 2</t>
+          <t>Algerian Ligue 2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exeter x Rotherham</t>
+          <t>USM El Harrach x Taghit</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Exeter</t>
+          <t>USM El Harrach</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rotherham</t>
+          <t>Taghit</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1089,14 +985,14 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>16.5</v>
+        <v>15</v>
       </c>
       <c r="K8" t="n">
-        <v>2.6</v>
+        <v>1.26</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>4-0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1115,21 +1011,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>229</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R8" t="n">
-        <v>200</v>
-      </c>
-      <c r="S8" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="T8" t="n">
-        <v>12.32</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9">
@@ -1140,32 +1022,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Scottish League One</t>
+          <t>Guatemalan Liga Nacional</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ross Co x Alloa</t>
+          <t>Deportivo Mixco x CSD Municipal</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ross Co</t>
+          <t>Deportivo Mixco</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Alloa</t>
+          <t>CSD Municipal</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1175,14 +1057,14 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>17.5</v>
       </c>
       <c r="K9" t="n">
-        <v>1.29</v>
+        <v>2.38</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>AO Home Win</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1201,21 +1083,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>229</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R9" t="n">
-        <v>200</v>
-      </c>
-      <c r="S9" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="T9" t="n">
-        <v>31.83</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10">
@@ -1226,32 +1094,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Scottish Championship</t>
+          <t>Brazilian Serie B</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Morton x Raith</t>
+          <t>Cuiaba x Ponte Preta</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Morton</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Raith</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1261,14 +1129,14 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>6.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>1.65</v>
+        <v>1.16</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1287,21 +1155,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>159</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R10" t="n">
-        <v>200</v>
-      </c>
-      <c r="S10" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="T10" t="n">
-        <v>35.37</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11">
@@ -1312,32 +1166,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>English National League</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Gateshead x Worthing</t>
+          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Gateshead</t>
+          <t>CSD Liniers de Ciudad Evita</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Worthing</t>
+          <t>Excursionistas</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1347,14 +1201,14 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="K11" t="n">
-        <v>1.5</v>
+        <v>1.01</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1373,21 +1227,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>231</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R11" t="n">
-        <v>200</v>
-      </c>
-      <c r="S11" t="n">
-        <v>32.26</v>
-      </c>
-      <c r="T11" t="n">
-        <v>30.81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -1398,32 +1238,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Algerian Ligue 2</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>USM El Harrach x Taghit</t>
+          <t>Camioneros x Deportivo Laferrere</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>USM El Harrach</t>
+          <t>Camioneros</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Taghit</t>
+          <t>Deportivo Laferrere</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1433,14 +1273,14 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>15</v>
+        <v>6.6</v>
       </c>
       <c r="K12" t="n">
-        <v>1.26</v>
+        <v>1.23</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1459,21 +1299,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R12" t="n">
-        <v>200</v>
-      </c>
-      <c r="S12" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="T12" t="n">
-        <v>13.65</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13">
@@ -1484,32 +1310,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>German Frauen-Bundesliga</t>
+          <t>Brazilian Serie C</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
+          <t>Floresta EC x Botafogo PB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W)</t>
+          <t>Floresta EC</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bayern Munich (W)</t>
+          <t>Botafogo PB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1519,14 +1345,14 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K13" t="n">
-        <v>1.58</v>
+        <v>1.48</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1545,21 +1371,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>12:55</t>
-        </is>
-      </c>
-      <c r="R13" t="n">
-        <v>200</v>
-      </c>
-      <c r="S13" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="T13" t="n">
-        <v>11.23</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14">
@@ -1570,32 +1382,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>German Frauen-Bundesliga</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W) x Bayern Munich (W)</t>
+          <t>Camioneros x Deportivo Laferrere</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt (W)</t>
+          <t>Camioneros</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bayern Munich (W)</t>
+          <t>Deportivo Laferrere</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1605,14 +1417,14 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="K14" t="n">
-        <v>1.58</v>
+        <v>1.02</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1631,21 +1443,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>12:55</t>
-        </is>
-      </c>
-      <c r="R14" t="n">
-        <v>200</v>
-      </c>
-      <c r="S14" t="n">
-        <v>40</v>
-      </c>
-      <c r="T14" t="n">
-        <v>38.2</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15">
@@ -1656,32 +1454,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Guatemalan Liga Nacional</t>
+          <t>Colombian Primera A</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Deportivo Mixco x CSD Municipal</t>
+          <t>Tolima x Boyaca Chico</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deportivo Mixco</t>
+          <t>Tolima</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>CSD Municipal</t>
+          <t>Boyaca Chico</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1691,10 +1489,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>17.5</v>
+        <v>6.4</v>
       </c>
       <c r="K15" t="n">
-        <v>2.38</v>
+        <v>1.28</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1703,7 +1501,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1717,21 +1515,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>141</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="R15" t="n">
-        <v>200</v>
-      </c>
-      <c r="S15" t="n">
-        <v>12.12</v>
-      </c>
-      <c r="T15" t="n">
-        <v>11.57</v>
+        <v>888</v>
       </c>
     </row>
     <row r="16">
@@ -1742,27 +1526,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>UEFA Nations League B</t>
+          <t>Bolivian Cup</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Switzerland x Slovenia</t>
+          <t>Nacional Potosi x CDT Real Oruro</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Nacional Potosi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>CDT Real Oruro</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1777,14 +1561,14 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="K16" t="n">
-        <v>1.36</v>
+        <v>1.32</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1803,21 +1587,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>91</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="R16" t="n">
-        <v>200</v>
-      </c>
-      <c r="S16" t="n">
-        <v>44.44</v>
-      </c>
-      <c r="T16" t="n">
-        <v>42.44</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17">
@@ -1828,32 +1598,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>UEFA Nations League B</t>
+          <t>Brazilian Serie C</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>North Macedonia x Scotland</t>
+          <t>Paysandu x Ferroviaria</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>Paysandu</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Ferroviaria</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1863,14 +1633,14 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>8.6</v>
+        <v>19</v>
       </c>
       <c r="K17" t="n">
-        <v>1.58</v>
+        <v>2.32</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1889,21 +1659,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>2784</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="R17" t="n">
-        <v>200</v>
-      </c>
-      <c r="S17" t="n">
-        <v>26.32</v>
-      </c>
-      <c r="T17" t="n">
-        <v>25.14</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
@@ -1914,32 +1670,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Brazilian Serie B</t>
+          <t>Chilean Primera B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Cuiaba x Ponte Preta</t>
+          <t>CD Santa Cruz x San Marcos</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>CD Santa Cruz</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>San Marcos</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1949,20 +1705,24 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>9.800000000000001</v>
+        <v>20</v>
       </c>
       <c r="K18" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
+        <v>2.64</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1971,21 +1731,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>97</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="R18" t="n">
-        <v>200</v>
-      </c>
-      <c r="S18" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="T18" t="n">
-        <v>21.71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19">
@@ -1996,32 +1742,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Argentinian Primera B Metropolitana</t>
+          <t>Colombian Cup</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
+          <t>Barranquilla x Millonarios</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CSD Liniers de Ciudad Evita</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Excursionistas</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2031,20 +1777,24 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>5</v>
+        <v>8.4</v>
       </c>
       <c r="K19" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2053,21 +1803,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>69</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="R19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S19" t="n">
-        <v>50</v>
-      </c>
-      <c r="T19" t="n">
-        <v>47.75</v>
+        <v>331</v>
       </c>
     </row>
     <row r="20">
@@ -2078,32 +1814,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Argentinian Primera B Metropolitana</t>
+          <t>Salvadoran Primera Division</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Camioneros x Deportivo Laferrere</t>
+          <t>Alianza FC (SLV) x CD Luis Angel Firpo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Camioneros</t>
+          <t>Alianza FC (SLV)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Deportivo Laferrere</t>
+          <t>CD Luis Angel Firpo</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2113,20 +1849,24 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>6.6</v>
+        <v>17</v>
       </c>
       <c r="K20" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
+        <v>2.82</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2135,349 +1875,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>282</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="R20" t="n">
-        <v>200</v>
-      </c>
-      <c r="S20" t="n">
-        <v>35.71</v>
-      </c>
-      <c r="T20" t="n">
-        <v>34.1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Brazilian Serie C</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Floresta EC x Botafogo PB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Floresta EC</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Botafogo PB</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>161</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="R21" t="n">
-        <v>200</v>
-      </c>
-      <c r="S21" t="n">
-        <v>10.81</v>
-      </c>
-      <c r="T21" t="n">
-        <v>10.32</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Argentinian Primera B Metropolitana</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Camioneros x Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Camioneros</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Deportivo Laferrere</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>18</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="R22" t="n">
-        <v>200</v>
-      </c>
-      <c r="S22" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="T22" t="n">
-        <v>11.23</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Colombian Primera A</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Tolima x Boyaca Chico</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Tolima</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Boyaca Chico</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="K23" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>888</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="R23" t="n">
-        <v>200</v>
-      </c>
-      <c r="S23" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="T23" t="n">
-        <v>35.37</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Bolivian Cup</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Nacional Potosi x CDT Real Oruro</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Nacional Potosi</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>CDT Real Oruro</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>7</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>170</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="R24" t="n">
-        <v>200</v>
-      </c>
-      <c r="S24" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="T24" t="n">
-        <v>31.83</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sinais): atualiza planilha de 03/10 com filtro de ligas perifericas (15 jogos, 14G/1R)
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-03.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -950,32 +950,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Algerian Ligue 2</t>
+          <t>Brazilian Serie B</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>USM El Harrach x Taghit</t>
+          <t>Cuiaba x Ponte Preta</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>USM El Harrach</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Taghit</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -985,14 +985,14 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>15</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>1.26</v>
+        <v>1.16</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9">
@@ -1022,32 +1022,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Guatemalan Liga Nacional</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Deportivo Mixco x CSD Municipal</t>
+          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Deportivo Mixco</t>
+          <t>CSD Liniers de Ciudad Evita</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CSD Municipal</t>
+          <t>Excursionistas</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1057,14 +1057,14 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
-        <v>2.38</v>
+        <v>1.01</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>141</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Brazilian Serie B</t>
+          <t>Argentinian Primera B Metropolitana</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cuiaba x Ponte Preta</t>
+          <t>Camioneros x Deportivo Laferrere</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Camioneros</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Deportivo Laferrere</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1129,14 +1129,14 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>9.800000000000001</v>
+        <v>6.6</v>
       </c>
       <c r="K10" t="n">
-        <v>1.16</v>
+        <v>1.23</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>97</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11">
@@ -1171,27 +1171,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Argentinian Primera B Metropolitana</t>
+          <t>Brazilian Serie C</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CSD Liniers de Ciudad Evita x Excursionistas</t>
+          <t>Floresta EC x Botafogo PB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CSD Liniers de Ciudad Evita</t>
+          <t>Floresta EC</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Excursionistas</t>
+          <t>Botafogo PB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1201,14 +1201,14 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>19.5</v>
       </c>
       <c r="K11" t="n">
-        <v>1.01</v>
+        <v>1.48</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>69</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1273,10 +1273,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>6.6</v>
+        <v>18</v>
       </c>
       <c r="K12" t="n">
-        <v>1.23</v>
+        <v>1.02</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>282</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13">
@@ -1310,32 +1310,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Brazilian Serie C</t>
+          <t>Colombian Primera A</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Floresta EC x Botafogo PB</t>
+          <t>Tolima x Boyaca Chico</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Floresta EC</t>
+          <t>Tolima</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Botafogo PB</t>
+          <t>Boyaca Chico</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1345,19 +1345,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>19.5</v>
+        <v>6.4</v>
       </c>
       <c r="K13" t="n">
-        <v>1.48</v>
+        <v>1.28</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>161</v>
+        <v>888</v>
       </c>
     </row>
     <row r="14">
@@ -1382,32 +1382,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Argentinian Primera B Metropolitana</t>
+          <t>Brazilian Serie C</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Camioneros x Deportivo Laferrere</t>
+          <t>Paysandu x Ferroviaria</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Camioneros</t>
+          <t>Paysandu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Deportivo Laferrere</t>
+          <t>Ferroviaria</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1417,14 +1417,14 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K14" t="n">
-        <v>1.02</v>
+        <v>2.32</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15">
@@ -1454,32 +1454,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Colombian Primera A</t>
+          <t>Chilean Primera B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tolima x Boyaca Chico</t>
+          <t>CD Santa Cruz x San Marcos</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tolima</t>
+          <t>CD Santa Cruz</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Boyaca Chico</t>
+          <t>San Marcos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1489,19 +1489,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>6.4</v>
+        <v>20</v>
       </c>
       <c r="K15" t="n">
-        <v>1.28</v>
+        <v>2.64</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>888</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16">
@@ -1526,32 +1526,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Bolivian Cup</t>
+          <t>Colombian Cup</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Nacional Potosi x CDT Real Oruro</t>
+          <t>Barranquilla x Millonarios</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nacional Potosi</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CDT Real Oruro</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1561,14 +1561,14 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>7</v>
+        <v>8.4</v>
       </c>
       <c r="K16" t="n">
-        <v>1.32</v>
+        <v>1.5</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1587,295 +1587,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Brazilian Serie C</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Paysandu x Ferroviaria</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Paysandu</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Ferroviaria</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>19</v>
-      </c>
-      <c r="K17" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>✅ LIQUIDADO</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Chilean Primera B</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>CD Santa Cruz x San Marcos</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>CD Santa Cruz</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>San Marcos</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>20</v>
-      </c>
-      <c r="K18" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>✅ LIQUIDADO</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>20:10</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Colombian Cup</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Barranquilla x Millonarios</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Barranquilla</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Millonarios</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="K19" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>✅ LIQUIDADO</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
         <v>331</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Salvadoran Primera Division</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Alianza FC (SLV) x CD Luis Angel Firpo</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Alianza FC (SLV)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>CD Luis Angel Firpo</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>17</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2-2</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>✅ LIQUIDADO</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>coletor (KO-10)</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>